<commit_message>
"atualização e manutenção do programa"
</commit_message>
<xml_diff>
--- a/Gerenciamento_lab.xlsx
+++ b/Gerenciamento_lab.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -525,6 +525,26 @@
         </is>
       </c>
       <c r="B11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>calcio</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ureia</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -539,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -608,6 +628,46 @@
           <t>Classificação:</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Absorbância teste direta:</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Absorbância teste total:</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Resultado direta:</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Resultado total:</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Resultado indireta:</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Classificação direta:</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Classificação total:</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Classificação indireta:</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -730,6 +790,94 @@
       <c r="M5" t="inlineStr">
         <is>
           <t>Desejável</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>18/08/2026 21:49:27</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>lucas</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>-0.07000000000000006</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.1139999999999999</v>
+      </c>
+      <c r="E6" t="n">
+        <v>42.98</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Dentro do valor de referência</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>18/08/2026 21:49:42</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>23459</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1231</v>
+      </c>
+      <c r="E7" t="n">
+        <v>190.57</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Fora dos padrões</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>18/08/2026 21:54:19</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>lucas</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.07000000000000006</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.1139999999999999</v>
+      </c>
+      <c r="E8" t="n">
+        <v>42.98245614035096</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Dentro do valor de referência</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
         </is>
       </c>
     </row>

</xml_diff>